<commit_message>
Add multi-agency support, barcode extraction, and parser enhancements
- Support JS Julfaqar Travels and Bharat Horizon Travels agency switching
- Auto-extract barcodes from uploaded PDFs with Code128 fallback
- Enhance ticket parser coverage across varied airline/OTA ticket formats
- Fix Fill Sample Ticket functionality in UI
- Clean up test/junk PDF files from workspace
</commit_message>
<xml_diff>
--- a/ticket_records.xlsx
+++ b/ticket_records.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bookings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -427,12 +427,12 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="49" customWidth="1" min="17" max="17"/>
     <col width="7" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -504,25 +504,20 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Payment Mode</t>
+          <t>Fare Type</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Fare Type</t>
+          <t>Refund Status</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Refund Status</t>
+          <t>Flight Status</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
-        <is>
-          <t>Flight Status</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -590,22 +585,22 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Non-Refundable</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Non-Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -671,22 +666,22 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -752,22 +747,22 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -833,22 +828,22 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -914,22 +909,22 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -995,22 +990,22 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1076,22 +1071,22 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Non-Refundable</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Non-Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1157,22 +1152,22 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Non-Refundable</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Non-Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1238,22 +1233,22 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -1319,22 +1314,22 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>STUDENT FARE</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>STUDENT FARE</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1400,22 +1395,22 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -1481,22 +1476,22 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -1562,22 +1557,22 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -1643,22 +1638,22 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1724,22 +1719,22 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1805,22 +1800,22 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -1881,22 +1876,22 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -1962,22 +1957,22 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Refundable</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via UPI</t>
         </is>
       </c>
     </row>
@@ -2043,22 +2038,22 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>REGULAR</t>
+          <t>Partially Refundable</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Partially Refundable</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Paid via Credit Card</t>
         </is>
       </c>
     </row>
@@ -2124,25 +2119,790 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>REGULAR</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Paid via UPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:06:34</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Refundable</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:07:25</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:07:58</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:17:04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:10:33</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Direct/Walk-in</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>JS89WQ</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>JS2026101401</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>MOHAMMAD JULFAQAR</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>+91 9825123456</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>STV → DEL</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Mon, 19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>09:15 AM</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>6E 5214</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>6550</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Thank you for booking with JS Julfaqar Travels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:23:22</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:27:01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Direct/Walk-in</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>JS89WQ</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>JS2026101401</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>MOHAMMAD JULFAQAR</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>+91 9825123456</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>STV → DEL</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Mon, 19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>6E 5214</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>6550</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Thank you for booking with JS Julfaqar Travels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:39:32</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:39:49</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:45:52</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>MAIN01</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MMT2605071001</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>JOHN DOE</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DEL → BLR</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Wed, 14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>6E 1234, 6E 5678</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>7200</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(parser): robust extraction for agency tickets (booking ID, baggage, 24h/12h times, wrapped surnames, single-digit flight numbers)
</commit_message>
<xml_diff>
--- a/ticket_records.xlsx
+++ b/ticket_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q372"/>
+  <dimension ref="A1:Q408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -27620,7 +27620,6 @@
           <t>Sun, 01 Nov 2026</t>
         </is>
       </c>
-      <c r="K372" t="inlineStr"/>
       <c r="L372" t="inlineStr">
         <is>
           <t>SG 5</t>
@@ -27644,7 +27643,2579 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="Q372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:40:18</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>JS JULFAQAR TRAVELS</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>27790166846</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>MD PARVEJ</t>
+        </is>
+      </c>
+      <c r="G373" t="n">
+        <v>1</v>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>+91 9601074574</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>IXB → HYD</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>IX 2893</t>
+        </is>
+      </c>
+      <c r="M373" t="n">
+        <v>20707</v>
+      </c>
+      <c r="N373" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P373" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:47:56</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>JS JULFAQAR TRAVELS</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>27790166846</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>MD PARVEJ</t>
+        </is>
+      </c>
+      <c r="G374" t="n">
+        <v>1</v>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>+91 9601074574</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>IXB → HYD</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>IX 2893</t>
+        </is>
+      </c>
+      <c r="M374" t="n">
+        <v>20707</v>
+      </c>
+      <c r="N374" t="inlineStr">
+        <is>
+          <t>SPECIAL FARE</t>
+        </is>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P374" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>2026-10-20 02:48:24</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>JS JULFAQAR TRAVELS</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>27790166846</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>MD PARVEJ</t>
+        </is>
+      </c>
+      <c r="G375" t="n">
+        <v>1</v>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>+91 9601074574</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M375" t="n">
+        <v>20707</v>
+      </c>
+      <c r="N375" t="inlineStr">
+        <is>
+          <t>SPECIAL FARE</t>
+        </is>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P375" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:12:17</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>JS JULFAQAR TRAVELS</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>FBB8S6XP</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>MD PARVEJ</t>
+        </is>
+      </c>
+      <c r="G376" t="n">
+        <v>1</v>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>+91 9601074574</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>IXB → HYD</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>IX 2893</t>
+        </is>
+      </c>
+      <c r="M376" t="n">
+        <v>20707</v>
+      </c>
+      <c r="N376" t="inlineStr">
+        <is>
+          <t>SPECIAL FARE</t>
+        </is>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P376" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:52</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Direct/Walk-in</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>75IDSB</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>BK75IDSB</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Lalita Verma</t>
+        </is>
+      </c>
+      <c r="G377" t="n">
+        <v>1</v>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>+91 9917342194</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>HBD → NNS</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Tue, 22 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>4H509</t>
+        </is>
+      </c>
+      <c r="M377" t="n">
+        <v>4725</v>
+      </c>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P377" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:53</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Direct/Walk-in</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>40BPCR</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>BK40BPCR</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Aditi Verma</t>
+        </is>
+      </c>
+      <c r="G378" t="n">
+        <v>2</v>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>+91 9149382841</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>HBD → NNS</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Fri, 16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>4H509</t>
+        </is>
+      </c>
+      <c r="M378" t="n">
+        <v>9450</v>
+      </c>
+      <c r="N378" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P378" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:53</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>YZ78TE</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>BKYZ78TE</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Mohammad Arif Salauddin</t>
+        </is>
+      </c>
+      <c r="G379" t="n">
+        <v>1</v>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>DEL → SHJ</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Wed, 30 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>IX 135</t>
+        </is>
+      </c>
+      <c r="M379" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N379" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P379" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:55</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>EKDZJR</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>27789896659</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Md Faruque Azam</t>
+        </is>
+      </c>
+      <c r="G380" t="n">
+        <v>1</v>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>DEL → DXB</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>SG 5</t>
+        </is>
+      </c>
+      <c r="M380" t="n">
+        <v>14842</v>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:57</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>AGUY2R</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>27595071738</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Pramod Agarwal</t>
+        </is>
+      </c>
+      <c r="G381" t="n">
+        <v>2</v>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>DEL → IXB</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Tue, 15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>6E 6124</t>
+        </is>
+      </c>
+      <c r="M381" t="n">
+        <v>9856</v>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>Partially Refundable</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:58</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>6BJHJR</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>GOFLISTANRR38067662</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Mohammad Firoz</t>
+        </is>
+      </c>
+      <c r="G382" t="n">
+        <v>1</v>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>AMD → SHJ</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Wed, 07 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>G9 419</t>
+        </is>
+      </c>
+      <c r="M382" t="n">
+        <v>13109</v>
+      </c>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P382" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:59</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Goibibo</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>AC5IJH</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>GOFLISTAO28H6547318</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Jugraj Singh</t>
+        </is>
+      </c>
+      <c r="G383" t="n">
+        <v>1</v>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>SHJ → ATQ</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>IX 138</t>
+        </is>
+      </c>
+      <c r="M383" t="n">
+        <v>22821</v>
+      </c>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P383" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:48:59</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Q32M6V</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>NN2ANXRB97552714085</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Shahwaz Shahwaz</t>
+        </is>
+      </c>
+      <c r="G384" t="n">
+        <v>1</v>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>IXB → SHJ</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Sat, 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>IX 1547, IX 251</t>
+        </is>
+      </c>
+      <c r="M384" t="n">
+        <v>14924</v>
+      </c>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P384" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:00</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Cleartrip</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>V3152V</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>CT1589766</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Md Parvej</t>
+        </is>
+      </c>
+      <c r="G385" t="n">
+        <v>5</v>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>+91 7759069422</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>BOM → SHJ</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Thu, 01 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>IX 251</t>
+        </is>
+      </c>
+      <c r="M385" t="n">
+        <v>84131.95</v>
+      </c>
+      <c r="N385" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P385" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:01</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Cleartrip</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>V3152V</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>CT1589766</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Md Parvej</t>
+        </is>
+      </c>
+      <c r="G386" t="n">
+        <v>5</v>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>BOM → SHJ</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Thu, 01 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>IX 251</t>
+        </is>
+      </c>
+      <c r="M386" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P386" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:01</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Cleartrip</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>V3152V</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>CT1589766</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Md Parvej</t>
+        </is>
+      </c>
+      <c r="G387" t="n">
+        <v>5</v>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>BOM → SHJ</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Thu, 01 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>IX 251</t>
+        </is>
+      </c>
+      <c r="M387" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P387" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:02</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Cleartrip</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>V3152V</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>CT1589766</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Md Parvej</t>
+        </is>
+      </c>
+      <c r="G388" t="n">
+        <v>5</v>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>+91 7759069422</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>BOM → SHJ</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Thu, 01 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>IX 251</t>
+        </is>
+      </c>
+      <c r="M388" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P388" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:02</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>WBMFPJ</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>CT1636212</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Sanjay Agarwal</t>
+        </is>
+      </c>
+      <c r="G389" t="n">
+        <v>3</v>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>+91 7759069422</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>DEL → IXB</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Thu, 05 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>6E 601</t>
+        </is>
+      </c>
+      <c r="M389" t="n">
+        <v>26567.1</v>
+      </c>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P389" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:03</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>I73JKV</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>NF2ANA9Z48042960338</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Sanyam Agarwal</t>
+        </is>
+      </c>
+      <c r="G390" t="n">
+        <v>3</v>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>IXB → DEL</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Sun, 06 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>6E 6125</t>
+        </is>
+      </c>
+      <c r="M390" t="n">
+        <v>11229</v>
+      </c>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>SAVER</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P390" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:03</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>8TFZ2W</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>NF9ANT3972086496191</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Aditi Verma</t>
+        </is>
+      </c>
+      <c r="G391" t="n">
+        <v>4</v>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>NNS → DED</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Thu, 01 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>9I 876</t>
+        </is>
+      </c>
+      <c r="M391" t="n">
+        <v>17476</v>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>SAVER</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P391" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:04</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>U3ZSGI</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>MN2TRVBLJVQ5M44G8095</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Shahid Alam</t>
+        </is>
+      </c>
+      <c r="G392" t="n">
+        <v>1</v>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>BOM → SHJ</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Sun, 04 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>IX 251</t>
+        </is>
+      </c>
+      <c r="M392" t="n">
+        <v>16500</v>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t>SPECIAL FARE</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:04</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>MakeMyTrip</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>KBCM9X</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>MN2LI5EQMZA0I6J59502</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Mohammad Adil Mohammad Imam</t>
+        </is>
+      </c>
+      <c r="G393" t="n">
+        <v>1</v>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>ATQ → SHJ</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Sat, 17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>IX 137</t>
+        </is>
+      </c>
+      <c r="M393" t="n">
+        <v>14499</v>
+      </c>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>SPECIAL FARE</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:25</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Flipkart</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>YDKKHA</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>260427555096</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Alka Agarwal</t>
+        </is>
+      </c>
+      <c r="G394" t="n">
+        <v>1</v>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>882 882 8282</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>GOX → IXB</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Mon, 04 May 2026</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>6E 945, 6E 149</t>
+        </is>
+      </c>
+      <c r="M394" t="n">
+        <v>8639</v>
+      </c>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P394" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:26</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>ACZW3X</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>27790349503</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Jatin Agarwal</t>
+        </is>
+      </c>
+      <c r="G395" t="n">
+        <v>1</v>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>IXB → DEL</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Wed, 21 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>QP 1808</t>
+        </is>
+      </c>
+      <c r="M395" t="n">
+        <v>5699</v>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>Partially Refundable</t>
+        </is>
+      </c>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>395</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:29</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>27790166846</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Mohammad Nurul</t>
+        </is>
+      </c>
+      <c r="G396" t="n">
+        <v>1</v>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M396" t="n">
+        <v>14707</v>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>Partially Refundable</t>
+        </is>
+      </c>
+      <c r="P396" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>396</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:30</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>NBY2QN</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>BKNBY2QN</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Navin Saraogi</t>
+        </is>
+      </c>
+      <c r="G397" t="n">
+        <v>5</v>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>+91-9832008383</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>GOX → IXB</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Thu, 10 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>IX 2764, IX 1081</t>
+        </is>
+      </c>
+      <c r="M397" t="n">
+        <v>56885</v>
+      </c>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P397" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>397</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:30</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Q32M6V</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>BKQ32M6V</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Shahwaz Shahwaz</t>
+        </is>
+      </c>
+      <c r="G398" t="n">
+        <v>1</v>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>+91-8789657048</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>IXB → SHJ</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Sat, 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>IX 1547, IX 251</t>
+        </is>
+      </c>
+      <c r="M398" t="n">
+        <v>18124</v>
+      </c>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>398</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:31</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Q32M6V</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>BKQ32M6V</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Shahwaz Shahwaz</t>
+        </is>
+      </c>
+      <c r="G399" t="n">
+        <v>1</v>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>+91-9601074574</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>IXB → SHJ</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Sat, 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>IX 1547, IX 251</t>
+        </is>
+      </c>
+      <c r="M399" t="n">
+        <v>18124</v>
+      </c>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>399</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:31</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Q32M6V</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>BKQ32M6V</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Shahwaz Shahwaz</t>
+        </is>
+      </c>
+      <c r="G400" t="n">
+        <v>1</v>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>+91-9601074574</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>IXB → SHJ</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Sat, 10 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>IX 1547, IX 251</t>
+        </is>
+      </c>
+      <c r="M400" t="n">
+        <v>18124</v>
+      </c>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P400" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>400</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:32</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>BKE3IFMF</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Mohammad Nurul</t>
+        </is>
+      </c>
+      <c r="G401" t="n">
+        <v>1</v>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>+91-8789657048</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M401" t="n">
+        <v>16341</v>
+      </c>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P401" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>401</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:35</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>DYFVMZ</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>BKDYFVMZ</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Himadri Mani</t>
+        </is>
+      </c>
+      <c r="G402" t="n">
+        <v>2</v>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>GOP → GOP</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Fri, 09 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>6E 2020, 6E 2019</t>
+        </is>
+      </c>
+      <c r="M402" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P402" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>402</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:35</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>A7BI8J</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>BKA7BI8J</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Saransh Sharma</t>
+        </is>
+      </c>
+      <c r="G403" t="n">
+        <v>1</v>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>+91 9876543210</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>BLR → DEL</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Fri, 01 May 2026</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>6E 6034</t>
+        </is>
+      </c>
+      <c r="M403" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="P403" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>403</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:36</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>AYKYHA</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>BKAYKYHA</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Absar Alam</t>
+        </is>
+      </c>
+      <c r="G404" t="n">
+        <v>1</v>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>+91-87******48</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>IXB → BOM</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Sun, 13 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>QP 1132</t>
+        </is>
+      </c>
+      <c r="M404" t="n">
+        <v>8548</v>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>SAVER</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P404" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>404</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:36</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>BKE3IFMF</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Mohammad Nurul</t>
+        </is>
+      </c>
+      <c r="G405" t="n">
+        <v>1</v>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>+91-8789657048</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M405" t="n">
+        <v>16341</v>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P405" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>405</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:37</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>PB16RA</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>FBB8S6XP</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>MOHAMMAD SHAMIM AKHTAR</t>
+        </is>
+      </c>
+      <c r="G406" t="n">
+        <v>2</v>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>+91-9217306715</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M406" t="n">
+        <v>34158.36</v>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>Refundable</t>
+        </is>
+      </c>
+      <c r="P406" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>406</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:40</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>E3IFMF</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>27790166846</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Mohammad Nurul</t>
+        </is>
+      </c>
+      <c r="G407" t="n">
+        <v>1</v>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>IXB → DXB</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>IX 2893, IX 969</t>
+        </is>
+      </c>
+      <c r="M407" t="n">
+        <v>14707</v>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>Partially Refundable</t>
+        </is>
+      </c>
+      <c r="P407" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>407</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026-10-20 03:49:41</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Paytm</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>EKDZJR</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>27789896659</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Md Faruque Azam</t>
+        </is>
+      </c>
+      <c r="G408" t="n">
+        <v>1</v>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>0120 4880880</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>DEL → DXB</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Sun, 01 Nov 2026</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr"/>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>SG 5</t>
+        </is>
+      </c>
+      <c r="M408" t="n">
+        <v>14842</v>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>Non-Refundable</t>
+        </is>
+      </c>
+      <c r="P408" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="Q408" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>